<commit_message>
[P2] chore(fixtures): regenerate planted-exception data and metric snapshots
tests/fixtures/tne_planted/data/*.xlsx: regenerated via generate.py from
this branch's plants.yaml (new B1/B2 plants and negatives, N2's stable
seed). tests/snapshots/surface2_results.json: regenerated via
orchestrator/eval/surface2.py -- every test still scores precision=1.0
recall=1.0 on the grown fixture. tests/snapshots/tne_real_metrics.json:
regenerated against synthetic_data/ -- the only real-data changes are
split_same_day_lines/split_window_lines replaced by split_groups/
split_lines (B3 metric rename), a new p_exp_hv population (N5, T4.4),
and t61d_pop/_dom row/amount counts shrinking as N5's amount > 0 filter
excludes credits (t61d_pop 136->133 rows, t61d_pop_dom 88->85 rows;
amounts rise since removing negative lines removes negative
contributions to the sum).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J4aRjEgFqM3dK34XuEwuYk
</commit_message>
<xml_diff>
--- a/tests/fixtures/tne_planted/data/Claims_Missing_Receipt_Affidavit.xlsx
+++ b/tests/fixtures/tne_planted/data/Claims_Missing_Receipt_Affidavit.xlsx
@@ -91,16 +91,16 @@
     <t>2025-09-01</t>
   </si>
   <si>
+    <t>Parking - Domestic Travel</t>
+  </si>
+  <si>
+    <t>Mobile Phone Charges</t>
+  </si>
+  <si>
     <t>Office Supplies</t>
   </si>
   <si>
-    <t>Parking - Domestic Travel</t>
-  </si>
-  <si>
     <t>Taxis - Domestic Travel</t>
-  </si>
-  <si>
-    <t>Mobile Phone Charges</t>
   </si>
   <si>
     <t>AUD</t>
@@ -473,19 +473,19 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2">
-        <v>90010</v>
+        <v>90001</v>
       </c>
       <c r="B2">
         <v>810000</v>
       </c>
       <c r="C2" s="1">
-        <v>46098</v>
+        <v>45693</v>
       </c>
       <c r="D2" t="s">
         <v>25</v>
       </c>
       <c r="E2">
-        <v>113.8</v>
+        <v>149.26</v>
       </c>
       <c r="F2" t="s">
         <v>29</v>
@@ -496,19 +496,19 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3">
-        <v>90006</v>
+        <v>90009</v>
       </c>
       <c r="B3">
         <v>810001</v>
       </c>
       <c r="C3" s="1">
-        <v>46033</v>
+        <v>46105</v>
       </c>
       <c r="D3" t="s">
         <v>26</v>
       </c>
       <c r="E3">
-        <v>310</v>
+        <v>76.3</v>
       </c>
       <c r="F3" t="s">
         <v>29</v>
@@ -519,25 +519,25 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4">
-        <v>90006</v>
+        <v>90004</v>
       </c>
       <c r="B4">
         <v>810002</v>
       </c>
       <c r="C4" s="1">
-        <v>45728</v>
+        <v>45867</v>
       </c>
       <c r="D4" t="s">
         <v>27</v>
       </c>
       <c r="E4">
-        <v>179.45</v>
+        <v>104.79</v>
       </c>
       <c r="F4" t="s">
         <v>29</v>
       </c>
       <c r="G4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -548,59 +548,59 @@
         <v>810003</v>
       </c>
       <c r="C5" s="1">
-        <v>45992</v>
+        <v>46084</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E5">
-        <v>89.41</v>
+        <v>261.66</v>
       </c>
       <c r="F5" t="s">
         <v>29</v>
       </c>
       <c r="G5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6">
-        <v>90002</v>
+        <v>90010</v>
       </c>
       <c r="B6">
         <v>810004</v>
       </c>
       <c r="C6" s="1">
-        <v>45663</v>
+        <v>45720</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E6">
-        <v>186.92</v>
+        <v>209.92</v>
       </c>
       <c r="F6" t="s">
         <v>29</v>
       </c>
       <c r="G6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7">
-        <v>90007</v>
+        <v>90008</v>
       </c>
       <c r="B7">
         <v>810005</v>
       </c>
       <c r="C7" s="1">
-        <v>45932</v>
+        <v>45766</v>
       </c>
       <c r="D7" t="s">
         <v>25</v>
       </c>
       <c r="E7">
-        <v>325.01</v>
+        <v>184.78</v>
       </c>
       <c r="F7" t="s">
         <v>29</v>
@@ -611,65 +611,65 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8">
-        <v>90011</v>
+        <v>90009</v>
       </c>
       <c r="B8">
         <v>810006</v>
       </c>
       <c r="C8" s="1">
-        <v>46075</v>
+        <v>45731</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E8">
-        <v>344.59</v>
+        <v>202.75</v>
       </c>
       <c r="F8" t="s">
         <v>29</v>
       </c>
       <c r="G8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9">
-        <v>90005</v>
+        <v>90002</v>
       </c>
       <c r="B9">
         <v>810007</v>
       </c>
       <c r="C9" s="1">
-        <v>46021</v>
+        <v>45982</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E9">
-        <v>320.89</v>
+        <v>334.85</v>
       </c>
       <c r="F9" t="s">
         <v>29</v>
       </c>
       <c r="G9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10">
-        <v>90009</v>
+        <v>90006</v>
       </c>
       <c r="B10">
         <v>810008</v>
       </c>
       <c r="C10" s="1">
-        <v>45673</v>
+        <v>46130</v>
       </c>
       <c r="D10" t="s">
         <v>26</v>
       </c>
       <c r="E10">
-        <v>219.52</v>
+        <v>190.51</v>
       </c>
       <c r="F10" t="s">
         <v>29</v>
@@ -680,19 +680,19 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11">
-        <v>90012</v>
+        <v>90008</v>
       </c>
       <c r="B11">
         <v>810009</v>
       </c>
       <c r="C11" s="1">
-        <v>45832</v>
+        <v>45870</v>
       </c>
       <c r="D11" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E11">
-        <v>36.21</v>
+        <v>111.15</v>
       </c>
       <c r="F11" t="s">
         <v>29</v>
@@ -703,65 +703,65 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12">
-        <v>90011</v>
+        <v>90007</v>
       </c>
       <c r="B12">
         <v>810010</v>
       </c>
       <c r="C12" s="1">
-        <v>46014</v>
+        <v>45696</v>
       </c>
       <c r="D12" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E12">
-        <v>52.01</v>
+        <v>18.86</v>
       </c>
       <c r="F12" t="s">
         <v>29</v>
       </c>
       <c r="G12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13">
-        <v>90012</v>
+        <v>90007</v>
       </c>
       <c r="B13">
         <v>810011</v>
       </c>
       <c r="C13" s="1">
-        <v>45785</v>
+        <v>45670</v>
       </c>
       <c r="D13" t="s">
         <v>27</v>
       </c>
       <c r="E13">
-        <v>219.15</v>
+        <v>34.77</v>
       </c>
       <c r="F13" t="s">
         <v>29</v>
       </c>
       <c r="G13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14">
-        <v>90009</v>
+        <v>90003</v>
       </c>
       <c r="B14">
         <v>810012</v>
       </c>
       <c r="C14" s="1">
-        <v>46127</v>
+        <v>46012</v>
       </c>
       <c r="D14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E14">
-        <v>166.93</v>
+        <v>247.19</v>
       </c>
       <c r="F14" t="s">
         <v>29</v>
@@ -772,19 +772,19 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15">
-        <v>90012</v>
+        <v>90006</v>
       </c>
       <c r="B15">
         <v>810013</v>
       </c>
       <c r="C15" s="1">
-        <v>45932</v>
+        <v>46042</v>
       </c>
       <c r="D15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E15">
-        <v>193.34</v>
+        <v>57.6</v>
       </c>
       <c r="F15" t="s">
         <v>29</v>
@@ -795,42 +795,42 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16">
-        <v>90001</v>
+        <v>90006</v>
       </c>
       <c r="B16">
         <v>810014</v>
       </c>
       <c r="C16" s="1">
-        <v>45928</v>
+        <v>45802</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E16">
-        <v>54.85</v>
+        <v>258.37</v>
       </c>
       <c r="F16" t="s">
         <v>29</v>
       </c>
       <c r="G16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17">
-        <v>90011</v>
+        <v>90003</v>
       </c>
       <c r="B17">
         <v>810015</v>
       </c>
       <c r="C17" s="1">
-        <v>45675</v>
+        <v>45780</v>
       </c>
       <c r="D17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E17">
-        <v>265.02</v>
+        <v>101.81</v>
       </c>
       <c r="F17" t="s">
         <v>29</v>
@@ -841,19 +841,19 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18">
-        <v>90010</v>
+        <v>90003</v>
       </c>
       <c r="B18">
         <v>810016</v>
       </c>
       <c r="C18" s="1">
-        <v>46085</v>
+        <v>45948</v>
       </c>
       <c r="D18" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E18">
-        <v>176.12</v>
+        <v>264.73</v>
       </c>
       <c r="F18" t="s">
         <v>29</v>
@@ -864,19 +864,19 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19">
-        <v>90001</v>
+        <v>90004</v>
       </c>
       <c r="B19">
         <v>810017</v>
       </c>
       <c r="C19" s="1">
-        <v>45796</v>
+        <v>46086</v>
       </c>
       <c r="D19" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E19">
-        <v>264.18</v>
+        <v>202.84</v>
       </c>
       <c r="F19" t="s">
         <v>29</v>
@@ -887,19 +887,19 @@
     </row>
     <row r="20" spans="1:7">
       <c r="A20">
-        <v>90005</v>
+        <v>90002</v>
       </c>
       <c r="B20">
         <v>810018</v>
       </c>
       <c r="C20" s="1">
-        <v>46006</v>
+        <v>46061</v>
       </c>
       <c r="D20" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E20">
-        <v>303.42</v>
+        <v>17.86</v>
       </c>
       <c r="F20" t="s">
         <v>29</v>
@@ -910,19 +910,19 @@
     </row>
     <row r="21" spans="1:7">
       <c r="A21">
-        <v>90010</v>
+        <v>90012</v>
       </c>
       <c r="B21">
         <v>810019</v>
       </c>
       <c r="C21" s="1">
-        <v>45757</v>
+        <v>45790</v>
       </c>
       <c r="D21" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E21">
-        <v>48.82</v>
+        <v>98.53</v>
       </c>
       <c r="F21" t="s">
         <v>29</v>
@@ -933,42 +933,42 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22">
-        <v>90011</v>
+        <v>90004</v>
       </c>
       <c r="B22">
         <v>810020</v>
       </c>
       <c r="C22" s="1">
-        <v>45774</v>
+        <v>45680</v>
       </c>
       <c r="D22" t="s">
         <v>26</v>
       </c>
       <c r="E22">
-        <v>60.59</v>
+        <v>131.45</v>
       </c>
       <c r="F22" t="s">
         <v>29</v>
       </c>
       <c r="G22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23">
-        <v>90002</v>
+        <v>90003</v>
       </c>
       <c r="B23">
         <v>810021</v>
       </c>
       <c r="C23" s="1">
-        <v>45744</v>
+        <v>45695</v>
       </c>
       <c r="D23" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E23">
-        <v>286.24</v>
+        <v>191.09</v>
       </c>
       <c r="F23" t="s">
         <v>29</v>
@@ -979,19 +979,19 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24">
-        <v>90001</v>
+        <v>90006</v>
       </c>
       <c r="B24">
         <v>810022</v>
       </c>
       <c r="C24" s="1">
-        <v>45826</v>
+        <v>45678</v>
       </c>
       <c r="D24" t="s">
         <v>27</v>
       </c>
       <c r="E24">
-        <v>339.22</v>
+        <v>245.59</v>
       </c>
       <c r="F24" t="s">
         <v>29</v>
@@ -1002,42 +1002,42 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25">
-        <v>90006</v>
+        <v>90009</v>
       </c>
       <c r="B25">
         <v>810023</v>
       </c>
       <c r="C25" s="1">
-        <v>45938</v>
+        <v>45927</v>
       </c>
       <c r="D25" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E25">
-        <v>83.90000000000001</v>
+        <v>145.29</v>
       </c>
       <c r="F25" t="s">
         <v>29</v>
       </c>
       <c r="G25" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26">
-        <v>90007</v>
+        <v>90009</v>
       </c>
       <c r="B26">
         <v>810024</v>
       </c>
       <c r="C26" s="1">
-        <v>46036</v>
+        <v>46025</v>
       </c>
       <c r="D26" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E26">
-        <v>135.88</v>
+        <v>242.19</v>
       </c>
       <c r="F26" t="s">
         <v>29</v>
@@ -1048,42 +1048,42 @@
     </row>
     <row r="27" spans="1:7">
       <c r="A27">
-        <v>90003</v>
+        <v>90010</v>
       </c>
       <c r="B27">
         <v>810025</v>
       </c>
       <c r="C27" s="1">
-        <v>45946</v>
+        <v>45866</v>
       </c>
       <c r="D27" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E27">
-        <v>119.72</v>
+        <v>278.14</v>
       </c>
       <c r="F27" t="s">
         <v>29</v>
       </c>
       <c r="G27" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28">
-        <v>90002</v>
+        <v>90007</v>
       </c>
       <c r="B28">
         <v>810026</v>
       </c>
       <c r="C28" s="1">
-        <v>45755</v>
+        <v>45688</v>
       </c>
       <c r="D28" t="s">
         <v>26</v>
       </c>
       <c r="E28">
-        <v>264.29</v>
+        <v>312.32</v>
       </c>
       <c r="F28" t="s">
         <v>29</v>
@@ -1094,48 +1094,48 @@
     </row>
     <row r="29" spans="1:7">
       <c r="A29">
-        <v>90011</v>
+        <v>90006</v>
       </c>
       <c r="B29">
         <v>810027</v>
       </c>
       <c r="C29" s="1">
-        <v>45832</v>
+        <v>45707</v>
       </c>
       <c r="D29" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E29">
-        <v>85.47</v>
+        <v>286.77</v>
       </c>
       <c r="F29" t="s">
         <v>29</v>
       </c>
       <c r="G29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30">
-        <v>90012</v>
+        <v>90010</v>
       </c>
       <c r="B30">
         <v>810028</v>
       </c>
       <c r="C30" s="1">
-        <v>45874</v>
+        <v>45729</v>
       </c>
       <c r="D30" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E30">
-        <v>201.6</v>
+        <v>302.14</v>
       </c>
       <c r="F30" t="s">
         <v>29</v>
       </c>
       <c r="G30" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -1146,13 +1146,13 @@
         <v>810029</v>
       </c>
       <c r="C31" s="1">
-        <v>45891</v>
+        <v>46103</v>
       </c>
       <c r="D31" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E31">
-        <v>254.73</v>
+        <v>334.08</v>
       </c>
       <c r="F31" t="s">
         <v>29</v>
@@ -1169,59 +1169,59 @@
         <v>810030</v>
       </c>
       <c r="C32" s="1">
-        <v>45825</v>
+        <v>45682</v>
       </c>
       <c r="D32" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E32">
-        <v>72.34999999999999</v>
+        <v>231.32</v>
       </c>
       <c r="F32" t="s">
         <v>29</v>
       </c>
       <c r="G32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:7">
       <c r="A33">
-        <v>90003</v>
+        <v>90008</v>
       </c>
       <c r="B33">
         <v>810031</v>
       </c>
       <c r="C33" s="1">
-        <v>46061</v>
+        <v>45908</v>
       </c>
       <c r="D33" t="s">
         <v>25</v>
       </c>
       <c r="E33">
-        <v>349.64</v>
+        <v>298.29</v>
       </c>
       <c r="F33" t="s">
         <v>29</v>
       </c>
       <c r="G33" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:7">
       <c r="A34">
-        <v>90012</v>
+        <v>90005</v>
       </c>
       <c r="B34">
         <v>810032</v>
       </c>
       <c r="C34" s="1">
-        <v>45661</v>
+        <v>45923</v>
       </c>
       <c r="D34" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E34">
-        <v>22.26</v>
+        <v>281.47</v>
       </c>
       <c r="F34" t="s">
         <v>29</v>
@@ -1232,48 +1232,48 @@
     </row>
     <row r="35" spans="1:7">
       <c r="A35">
-        <v>90011</v>
+        <v>90006</v>
       </c>
       <c r="B35">
         <v>810033</v>
       </c>
       <c r="C35" s="1">
-        <v>46131</v>
+        <v>45886</v>
       </c>
       <c r="D35" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E35">
-        <v>127.45</v>
+        <v>333.5</v>
       </c>
       <c r="F35" t="s">
         <v>29</v>
       </c>
       <c r="G35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="A36">
-        <v>90010</v>
+        <v>90009</v>
       </c>
       <c r="B36">
         <v>810034</v>
       </c>
       <c r="C36" s="1">
-        <v>46077</v>
+        <v>45803</v>
       </c>
       <c r="D36" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E36">
-        <v>325.93</v>
+        <v>144.62</v>
       </c>
       <c r="F36" t="s">
         <v>29</v>
       </c>
       <c r="G36" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -1284,13 +1284,13 @@
         <v>810035</v>
       </c>
       <c r="C37" s="1">
-        <v>45963</v>
+        <v>45777</v>
       </c>
       <c r="D37" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E37">
-        <v>158.48</v>
+        <v>184.86</v>
       </c>
       <c r="F37" t="s">
         <v>29</v>
@@ -1301,42 +1301,42 @@
     </row>
     <row r="38" spans="1:7">
       <c r="A38">
-        <v>90005</v>
+        <v>90010</v>
       </c>
       <c r="B38">
         <v>810036</v>
       </c>
       <c r="C38" s="1">
-        <v>45961</v>
+        <v>45775</v>
       </c>
       <c r="D38" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E38">
-        <v>318.61</v>
+        <v>116.51</v>
       </c>
       <c r="F38" t="s">
         <v>29</v>
       </c>
       <c r="G38" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39">
-        <v>90001</v>
+        <v>90012</v>
       </c>
       <c r="B39">
         <v>810037</v>
       </c>
       <c r="C39" s="1">
-        <v>45920</v>
+        <v>46127</v>
       </c>
       <c r="D39" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E39">
-        <v>341.68</v>
+        <v>240.53</v>
       </c>
       <c r="F39" t="s">
         <v>29</v>
@@ -1347,19 +1347,19 @@
     </row>
     <row r="40" spans="1:7">
       <c r="A40">
-        <v>90007</v>
+        <v>90010</v>
       </c>
       <c r="B40">
         <v>810038</v>
       </c>
       <c r="C40" s="1">
-        <v>45917</v>
+        <v>45974</v>
       </c>
       <c r="D40" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E40">
-        <v>316.8</v>
+        <v>95.56999999999999</v>
       </c>
       <c r="F40" t="s">
         <v>29</v>
@@ -1376,13 +1376,13 @@
         <v>810039</v>
       </c>
       <c r="C41" s="1">
-        <v>46054</v>
+        <v>45879</v>
       </c>
       <c r="D41" t="s">
         <v>25</v>
       </c>
       <c r="E41">
-        <v>299.82</v>
+        <v>239.57</v>
       </c>
       <c r="F41" t="s">
         <v>29</v>
@@ -1399,13 +1399,13 @@
         <v>810040</v>
       </c>
       <c r="C42" s="1">
-        <v>45749</v>
+        <v>45685</v>
       </c>
       <c r="D42" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E42">
-        <v>274.59</v>
+        <v>116.09</v>
       </c>
       <c r="F42" t="s">
         <v>29</v>
@@ -1416,42 +1416,42 @@
     </row>
     <row r="43" spans="1:7">
       <c r="A43">
-        <v>90009</v>
+        <v>90010</v>
       </c>
       <c r="B43">
         <v>810041</v>
       </c>
       <c r="C43" s="1">
-        <v>45866</v>
+        <v>45953</v>
       </c>
       <c r="D43" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E43">
-        <v>198.51</v>
+        <v>174.19</v>
       </c>
       <c r="F43" t="s">
         <v>29</v>
       </c>
       <c r="G43" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:7">
       <c r="A44">
-        <v>90007</v>
+        <v>90010</v>
       </c>
       <c r="B44">
         <v>810042</v>
       </c>
       <c r="C44" s="1">
-        <v>46117</v>
+        <v>45909</v>
       </c>
       <c r="D44" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E44">
-        <v>17.2</v>
+        <v>169.95</v>
       </c>
       <c r="F44" t="s">
         <v>29</v>
@@ -1462,19 +1462,19 @@
     </row>
     <row r="45" spans="1:7">
       <c r="A45">
-        <v>90005</v>
+        <v>90008</v>
       </c>
       <c r="B45">
         <v>810043</v>
       </c>
       <c r="C45" s="1">
-        <v>45765</v>
+        <v>45942</v>
       </c>
       <c r="D45" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E45">
-        <v>194.33</v>
+        <v>117.4</v>
       </c>
       <c r="F45" t="s">
         <v>29</v>
@@ -1485,19 +1485,19 @@
     </row>
     <row r="46" spans="1:7">
       <c r="A46">
-        <v>90006</v>
+        <v>90004</v>
       </c>
       <c r="B46">
         <v>810044</v>
       </c>
       <c r="C46" s="1">
-        <v>45883</v>
+        <v>45804</v>
       </c>
       <c r="D46" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E46">
-        <v>167.36</v>
+        <v>286.26</v>
       </c>
       <c r="F46" t="s">
         <v>29</v>
@@ -1508,19 +1508,19 @@
     </row>
     <row r="47" spans="1:7">
       <c r="A47">
-        <v>90008</v>
+        <v>90011</v>
       </c>
       <c r="B47">
         <v>810045</v>
       </c>
       <c r="C47" s="1">
-        <v>45707</v>
+        <v>45730</v>
       </c>
       <c r="D47" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E47">
-        <v>332.52</v>
+        <v>228.6</v>
       </c>
       <c r="F47" t="s">
         <v>29</v>
@@ -1531,19 +1531,19 @@
     </row>
     <row r="48" spans="1:7">
       <c r="A48">
-        <v>90010</v>
+        <v>90002</v>
       </c>
       <c r="B48">
         <v>810046</v>
       </c>
       <c r="C48" s="1">
-        <v>45684</v>
+        <v>46117</v>
       </c>
       <c r="D48" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E48">
-        <v>93.17</v>
+        <v>141.76</v>
       </c>
       <c r="F48" t="s">
         <v>29</v>
@@ -1554,19 +1554,19 @@
     </row>
     <row r="49" spans="1:7">
       <c r="A49">
-        <v>90001</v>
+        <v>90010</v>
       </c>
       <c r="B49">
         <v>810047</v>
       </c>
       <c r="C49" s="1">
-        <v>46017</v>
+        <v>45791</v>
       </c>
       <c r="D49" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E49">
-        <v>24.75</v>
+        <v>251.54</v>
       </c>
       <c r="F49" t="s">
         <v>29</v>
@@ -1577,19 +1577,19 @@
     </row>
     <row r="50" spans="1:7">
       <c r="A50">
-        <v>90006</v>
+        <v>90004</v>
       </c>
       <c r="B50">
         <v>810048</v>
       </c>
       <c r="C50" s="1">
-        <v>45705</v>
+        <v>45680</v>
       </c>
       <c r="D50" t="s">
         <v>25</v>
       </c>
       <c r="E50">
-        <v>172.43</v>
+        <v>22.95</v>
       </c>
       <c r="F50" t="s">
         <v>29</v>
@@ -1600,25 +1600,25 @@
     </row>
     <row r="51" spans="1:7">
       <c r="A51">
-        <v>90008</v>
+        <v>90012</v>
       </c>
       <c r="B51">
         <v>810049</v>
       </c>
       <c r="C51" s="1">
-        <v>46020</v>
+        <v>45691</v>
       </c>
       <c r="D51" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E51">
-        <v>270.77</v>
+        <v>183.38</v>
       </c>
       <c r="F51" t="s">
         <v>29</v>
       </c>
       <c r="G51" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -1629,42 +1629,42 @@
         <v>810050</v>
       </c>
       <c r="C52" s="1">
-        <v>45661</v>
+        <v>45761</v>
       </c>
       <c r="D52" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E52">
-        <v>208.45</v>
+        <v>169.95</v>
       </c>
       <c r="F52" t="s">
         <v>29</v>
       </c>
       <c r="G52" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="53" spans="1:7">
       <c r="A53">
-        <v>90011</v>
+        <v>90009</v>
       </c>
       <c r="B53">
         <v>810051</v>
       </c>
       <c r="C53" s="1">
-        <v>45985</v>
+        <v>45842</v>
       </c>
       <c r="D53" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E53">
-        <v>316.87</v>
+        <v>113.12</v>
       </c>
       <c r="F53" t="s">
         <v>29</v>
       </c>
       <c r="G53" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -1675,36 +1675,36 @@
         <v>810052</v>
       </c>
       <c r="C54" s="1">
-        <v>45943</v>
+        <v>45791</v>
       </c>
       <c r="D54" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E54">
-        <v>226.64</v>
+        <v>78.16</v>
       </c>
       <c r="F54" t="s">
         <v>29</v>
       </c>
       <c r="G54" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="55" spans="1:7">
       <c r="A55">
-        <v>90004</v>
+        <v>90012</v>
       </c>
       <c r="B55">
         <v>810053</v>
       </c>
       <c r="C55" s="1">
-        <v>46089</v>
+        <v>45824</v>
       </c>
       <c r="D55" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E55">
-        <v>246.42</v>
+        <v>133.96</v>
       </c>
       <c r="F55" t="s">
         <v>29</v>
@@ -1715,19 +1715,19 @@
     </row>
     <row r="56" spans="1:7">
       <c r="A56">
-        <v>90005</v>
+        <v>90010</v>
       </c>
       <c r="B56">
         <v>810054</v>
       </c>
       <c r="C56" s="1">
-        <v>45910</v>
+        <v>45978</v>
       </c>
       <c r="D56" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E56">
-        <v>337.08</v>
+        <v>171.03</v>
       </c>
       <c r="F56" t="s">
         <v>29</v>
@@ -1738,19 +1738,19 @@
     </row>
     <row r="57" spans="1:7">
       <c r="A57">
-        <v>90005</v>
+        <v>90009</v>
       </c>
       <c r="B57">
         <v>810055</v>
       </c>
       <c r="C57" s="1">
-        <v>46113</v>
+        <v>45667</v>
       </c>
       <c r="D57" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E57">
-        <v>190.58</v>
+        <v>224.35</v>
       </c>
       <c r="F57" t="s">
         <v>29</v>
@@ -1761,19 +1761,19 @@
     </row>
     <row r="58" spans="1:7">
       <c r="A58">
-        <v>90004</v>
+        <v>90012</v>
       </c>
       <c r="B58">
         <v>810056</v>
       </c>
       <c r="C58" s="1">
-        <v>45743</v>
+        <v>46002</v>
       </c>
       <c r="D58" t="s">
         <v>25</v>
       </c>
       <c r="E58">
-        <v>76.45</v>
+        <v>94.70999999999999</v>
       </c>
       <c r="F58" t="s">
         <v>29</v>
@@ -1784,65 +1784,65 @@
     </row>
     <row r="59" spans="1:7">
       <c r="A59">
-        <v>90003</v>
+        <v>90010</v>
       </c>
       <c r="B59">
         <v>810057</v>
       </c>
       <c r="C59" s="1">
-        <v>45778</v>
+        <v>46007</v>
       </c>
       <c r="D59" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E59">
-        <v>78.76000000000001</v>
+        <v>208.22</v>
       </c>
       <c r="F59" t="s">
         <v>29</v>
       </c>
       <c r="G59" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="60" spans="1:7">
       <c r="A60">
-        <v>90009</v>
+        <v>90010</v>
       </c>
       <c r="B60">
         <v>810058</v>
       </c>
       <c r="C60" s="1">
-        <v>45947</v>
+        <v>46002</v>
       </c>
       <c r="D60" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E60">
-        <v>242.48</v>
+        <v>20.59</v>
       </c>
       <c r="F60" t="s">
         <v>29</v>
       </c>
       <c r="G60" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="61" spans="1:7">
       <c r="A61">
-        <v>90010</v>
+        <v>90006</v>
       </c>
       <c r="B61">
         <v>810059</v>
       </c>
       <c r="C61" s="1">
-        <v>45661</v>
+        <v>45830</v>
       </c>
       <c r="D61" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E61">
-        <v>156.34</v>
+        <v>204.94</v>
       </c>
       <c r="F61" t="s">
         <v>29</v>
@@ -1853,19 +1853,19 @@
     </row>
     <row r="62" spans="1:7">
       <c r="A62">
-        <v>90012</v>
+        <v>90008</v>
       </c>
       <c r="B62">
         <v>810060</v>
       </c>
       <c r="C62" s="1">
-        <v>45903</v>
+        <v>46138</v>
       </c>
       <c r="D62" t="s">
         <v>28</v>
       </c>
       <c r="E62">
-        <v>298.08</v>
+        <v>295.68</v>
       </c>
       <c r="F62" t="s">
         <v>29</v>
@@ -1876,42 +1876,42 @@
     </row>
     <row r="63" spans="1:7">
       <c r="A63">
-        <v>90009</v>
+        <v>90007</v>
       </c>
       <c r="B63">
         <v>810061</v>
       </c>
       <c r="C63" s="1">
-        <v>45830</v>
+        <v>45932</v>
       </c>
       <c r="D63" t="s">
         <v>28</v>
       </c>
       <c r="E63">
-        <v>208.8</v>
+        <v>243.33</v>
       </c>
       <c r="F63" t="s">
         <v>29</v>
       </c>
       <c r="G63" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="64" spans="1:7">
       <c r="A64">
-        <v>90005</v>
+        <v>90002</v>
       </c>
       <c r="B64">
         <v>810062</v>
       </c>
       <c r="C64" s="1">
-        <v>45706</v>
+        <v>45784</v>
       </c>
       <c r="D64" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E64">
-        <v>57.79</v>
+        <v>340.35</v>
       </c>
       <c r="F64" t="s">
         <v>29</v>
@@ -1922,42 +1922,42 @@
     </row>
     <row r="65" spans="1:7">
       <c r="A65">
-        <v>90006</v>
+        <v>90012</v>
       </c>
       <c r="B65">
         <v>810063</v>
       </c>
       <c r="C65" s="1">
-        <v>45788</v>
+        <v>45681</v>
       </c>
       <c r="D65" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E65">
-        <v>173.27</v>
+        <v>201.54</v>
       </c>
       <c r="F65" t="s">
         <v>29</v>
       </c>
       <c r="G65" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="66" spans="1:7">
       <c r="A66">
-        <v>90009</v>
+        <v>90005</v>
       </c>
       <c r="B66">
         <v>810064</v>
       </c>
       <c r="C66" s="1">
-        <v>45960</v>
+        <v>45663</v>
       </c>
       <c r="D66" t="s">
         <v>25</v>
       </c>
       <c r="E66">
-        <v>83.75</v>
+        <v>192.53</v>
       </c>
       <c r="F66" t="s">
         <v>29</v>
@@ -1968,65 +1968,65 @@
     </row>
     <row r="67" spans="1:7">
       <c r="A67">
-        <v>90004</v>
+        <v>90009</v>
       </c>
       <c r="B67">
         <v>810065</v>
       </c>
       <c r="C67" s="1">
-        <v>46103</v>
+        <v>46016</v>
       </c>
       <c r="D67" t="s">
         <v>27</v>
       </c>
       <c r="E67">
-        <v>163.85</v>
+        <v>223.26</v>
       </c>
       <c r="F67" t="s">
         <v>29</v>
       </c>
       <c r="G67" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="68" spans="1:7">
       <c r="A68">
-        <v>90005</v>
+        <v>90010</v>
       </c>
       <c r="B68">
         <v>810066</v>
       </c>
       <c r="C68" s="1">
-        <v>46013</v>
+        <v>46124</v>
       </c>
       <c r="D68" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E68">
-        <v>185.57</v>
+        <v>181.31</v>
       </c>
       <c r="F68" t="s">
         <v>29</v>
       </c>
       <c r="G68" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="69" spans="1:7">
       <c r="A69">
-        <v>90009</v>
+        <v>90007</v>
       </c>
       <c r="B69">
         <v>810067</v>
       </c>
       <c r="C69" s="1">
-        <v>45759</v>
+        <v>45889</v>
       </c>
       <c r="D69" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E69">
-        <v>259.39</v>
+        <v>347.06</v>
       </c>
       <c r="F69" t="s">
         <v>29</v>
@@ -2037,19 +2037,19 @@
     </row>
     <row r="70" spans="1:7">
       <c r="A70">
-        <v>90009</v>
+        <v>90008</v>
       </c>
       <c r="B70">
         <v>810068</v>
       </c>
       <c r="C70" s="1">
-        <v>46094</v>
+        <v>45822</v>
       </c>
       <c r="D70" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E70">
-        <v>118.42</v>
+        <v>298.97</v>
       </c>
       <c r="F70" t="s">
         <v>29</v>
@@ -2060,111 +2060,111 @@
     </row>
     <row r="71" spans="1:7">
       <c r="A71">
-        <v>90009</v>
+        <v>90001</v>
       </c>
       <c r="B71">
         <v>810069</v>
       </c>
       <c r="C71" s="1">
-        <v>45846</v>
+        <v>45900</v>
       </c>
       <c r="D71" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E71">
-        <v>317.03</v>
+        <v>144.12</v>
       </c>
       <c r="F71" t="s">
         <v>29</v>
       </c>
       <c r="G71" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="72" spans="1:7">
       <c r="A72">
-        <v>90010</v>
+        <v>90009</v>
       </c>
       <c r="B72">
         <v>810070</v>
       </c>
       <c r="C72" s="1">
-        <v>45886</v>
+        <v>46034</v>
       </c>
       <c r="D72" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E72">
-        <v>188.33</v>
+        <v>302.73</v>
       </c>
       <c r="F72" t="s">
         <v>29</v>
       </c>
       <c r="G72" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="73" spans="1:7">
       <c r="A73">
-        <v>90008</v>
+        <v>90003</v>
       </c>
       <c r="B73">
         <v>810071</v>
       </c>
       <c r="C73" s="1">
-        <v>46107</v>
+        <v>45676</v>
       </c>
       <c r="D73" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E73">
-        <v>93.98</v>
+        <v>51.04</v>
       </c>
       <c r="F73" t="s">
         <v>29</v>
       </c>
       <c r="G73" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="74" spans="1:7">
       <c r="A74">
-        <v>90004</v>
+        <v>90012</v>
       </c>
       <c r="B74">
         <v>810072</v>
       </c>
       <c r="C74" s="1">
-        <v>45773</v>
+        <v>46126</v>
       </c>
       <c r="D74" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E74">
-        <v>250.79</v>
+        <v>83.66</v>
       </c>
       <c r="F74" t="s">
         <v>29</v>
       </c>
       <c r="G74" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="75" spans="1:7">
       <c r="A75">
-        <v>90008</v>
+        <v>90002</v>
       </c>
       <c r="B75">
         <v>810073</v>
       </c>
       <c r="C75" s="1">
-        <v>46123</v>
+        <v>45937</v>
       </c>
       <c r="D75" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E75">
-        <v>206.86</v>
+        <v>228.05</v>
       </c>
       <c r="F75" t="s">
         <v>29</v>
@@ -2175,25 +2175,25 @@
     </row>
     <row r="76" spans="1:7">
       <c r="A76">
-        <v>90012</v>
+        <v>90001</v>
       </c>
       <c r="B76">
         <v>810074</v>
       </c>
       <c r="C76" s="1">
-        <v>45855</v>
+        <v>45956</v>
       </c>
       <c r="D76" t="s">
         <v>26</v>
       </c>
       <c r="E76">
-        <v>250.86</v>
+        <v>49.51</v>
       </c>
       <c r="F76" t="s">
         <v>29</v>
       </c>
       <c r="G76" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="77" spans="1:7">
@@ -2204,36 +2204,36 @@
         <v>810075</v>
       </c>
       <c r="C77" s="1">
-        <v>45687</v>
+        <v>45920</v>
       </c>
       <c r="D77" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E77">
-        <v>246.23</v>
+        <v>62.96</v>
       </c>
       <c r="F77" t="s">
         <v>29</v>
       </c>
       <c r="G77" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="78" spans="1:7">
       <c r="A78">
-        <v>90010</v>
+        <v>90006</v>
       </c>
       <c r="B78">
         <v>810076</v>
       </c>
       <c r="C78" s="1">
-        <v>46065</v>
+        <v>45836</v>
       </c>
       <c r="D78" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E78">
-        <v>174.6</v>
+        <v>225.45</v>
       </c>
       <c r="F78" t="s">
         <v>29</v>
@@ -2244,19 +2244,19 @@
     </row>
     <row r="79" spans="1:7">
       <c r="A79">
-        <v>90002</v>
+        <v>90005</v>
       </c>
       <c r="B79">
         <v>810077</v>
       </c>
       <c r="C79" s="1">
-        <v>46006</v>
+        <v>45921</v>
       </c>
       <c r="D79" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E79">
-        <v>142.45</v>
+        <v>163.48</v>
       </c>
       <c r="F79" t="s">
         <v>29</v>
@@ -2267,19 +2267,19 @@
     </row>
     <row r="80" spans="1:7">
       <c r="A80">
-        <v>90007</v>
+        <v>90008</v>
       </c>
       <c r="B80">
         <v>810078</v>
       </c>
       <c r="C80" s="1">
-        <v>45720</v>
+        <v>45867</v>
       </c>
       <c r="D80" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E80">
-        <v>66.31999999999999</v>
+        <v>252.04</v>
       </c>
       <c r="F80" t="s">
         <v>29</v>
@@ -2290,65 +2290,65 @@
     </row>
     <row r="81" spans="1:7">
       <c r="A81">
-        <v>90010</v>
+        <v>90003</v>
       </c>
       <c r="B81">
         <v>810079</v>
       </c>
       <c r="C81" s="1">
-        <v>46057</v>
+        <v>45710</v>
       </c>
       <c r="D81" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E81">
-        <v>144.53</v>
+        <v>190.13</v>
       </c>
       <c r="F81" t="s">
         <v>29</v>
       </c>
       <c r="G81" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="82" spans="1:7">
       <c r="A82">
-        <v>90007</v>
+        <v>90003</v>
       </c>
       <c r="B82">
         <v>810080</v>
       </c>
       <c r="C82" s="1">
-        <v>46002</v>
+        <v>45925</v>
       </c>
       <c r="D82" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E82">
-        <v>241.77</v>
+        <v>273.13</v>
       </c>
       <c r="F82" t="s">
         <v>29</v>
       </c>
       <c r="G82" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="83" spans="1:7">
       <c r="A83">
-        <v>90005</v>
+        <v>90007</v>
       </c>
       <c r="B83">
         <v>810081</v>
       </c>
       <c r="C83" s="1">
-        <v>45999</v>
+        <v>45771</v>
       </c>
       <c r="D83" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E83">
-        <v>312.71</v>
+        <v>222.01</v>
       </c>
       <c r="F83" t="s">
         <v>29</v>
@@ -2359,65 +2359,65 @@
     </row>
     <row r="84" spans="1:7">
       <c r="A84">
-        <v>90006</v>
+        <v>90008</v>
       </c>
       <c r="B84">
         <v>810082</v>
       </c>
       <c r="C84" s="1">
-        <v>45755</v>
+        <v>45967</v>
       </c>
       <c r="D84" t="s">
         <v>27</v>
       </c>
       <c r="E84">
-        <v>55.9</v>
+        <v>265.56</v>
       </c>
       <c r="F84" t="s">
         <v>29</v>
       </c>
       <c r="G84" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="85" spans="1:7">
       <c r="A85">
-        <v>90003</v>
+        <v>90004</v>
       </c>
       <c r="B85">
         <v>810083</v>
       </c>
       <c r="C85" s="1">
-        <v>45852</v>
+        <v>45729</v>
       </c>
       <c r="D85" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E85">
-        <v>295.02</v>
+        <v>265.96</v>
       </c>
       <c r="F85" t="s">
         <v>29</v>
       </c>
       <c r="G85" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="86" spans="1:7">
       <c r="A86">
-        <v>90006</v>
+        <v>90003</v>
       </c>
       <c r="B86">
         <v>810084</v>
       </c>
       <c r="C86" s="1">
-        <v>46021</v>
+        <v>45900</v>
       </c>
       <c r="D86" t="s">
         <v>28</v>
       </c>
       <c r="E86">
-        <v>120.86</v>
+        <v>151.6</v>
       </c>
       <c r="F86" t="s">
         <v>29</v>
@@ -2428,42 +2428,42 @@
     </row>
     <row r="87" spans="1:7">
       <c r="A87">
-        <v>90003</v>
+        <v>90012</v>
       </c>
       <c r="B87">
         <v>810085</v>
       </c>
       <c r="C87" s="1">
-        <v>46119</v>
+        <v>46044</v>
       </c>
       <c r="D87" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E87">
-        <v>132.58</v>
+        <v>31.27</v>
       </c>
       <c r="F87" t="s">
         <v>29</v>
       </c>
       <c r="G87" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="88" spans="1:7">
       <c r="A88">
-        <v>90012</v>
+        <v>90005</v>
       </c>
       <c r="B88">
         <v>810086</v>
       </c>
       <c r="C88" s="1">
-        <v>46094</v>
+        <v>45851</v>
       </c>
       <c r="D88" t="s">
         <v>28</v>
       </c>
       <c r="E88">
-        <v>82.2</v>
+        <v>127.46</v>
       </c>
       <c r="F88" t="s">
         <v>29</v>
@@ -2474,19 +2474,19 @@
     </row>
     <row r="89" spans="1:7">
       <c r="A89">
-        <v>90011</v>
+        <v>90009</v>
       </c>
       <c r="B89">
         <v>810087</v>
       </c>
       <c r="C89" s="1">
-        <v>45892</v>
+        <v>45994</v>
       </c>
       <c r="D89" t="s">
         <v>27</v>
       </c>
       <c r="E89">
-        <v>236.37</v>
+        <v>261.34</v>
       </c>
       <c r="F89" t="s">
         <v>29</v>
@@ -2497,19 +2497,19 @@
     </row>
     <row r="90" spans="1:7">
       <c r="A90">
-        <v>90012</v>
+        <v>90010</v>
       </c>
       <c r="B90">
         <v>810088</v>
       </c>
       <c r="C90" s="1">
-        <v>45729</v>
+        <v>45912</v>
       </c>
       <c r="D90" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E90">
-        <v>81.56999999999999</v>
+        <v>174.26</v>
       </c>
       <c r="F90" t="s">
         <v>29</v>
@@ -2520,19 +2520,19 @@
     </row>
     <row r="91" spans="1:7">
       <c r="A91">
-        <v>90011</v>
+        <v>90005</v>
       </c>
       <c r="B91">
         <v>810089</v>
       </c>
       <c r="C91" s="1">
-        <v>46080</v>
+        <v>45780</v>
       </c>
       <c r="D91" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E91">
-        <v>214.11</v>
+        <v>50.75</v>
       </c>
       <c r="F91" t="s">
         <v>29</v>
@@ -2543,19 +2543,19 @@
     </row>
     <row r="92" spans="1:7">
       <c r="A92">
-        <v>90003</v>
+        <v>90009</v>
       </c>
       <c r="B92">
         <v>810090</v>
       </c>
       <c r="C92" s="1">
-        <v>45670</v>
+        <v>46068</v>
       </c>
       <c r="D92" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E92">
-        <v>295.43</v>
+        <v>171.22</v>
       </c>
       <c r="F92" t="s">
         <v>29</v>
@@ -2566,19 +2566,19 @@
     </row>
     <row r="93" spans="1:7">
       <c r="A93">
-        <v>90008</v>
+        <v>90007</v>
       </c>
       <c r="B93">
         <v>810091</v>
       </c>
       <c r="C93" s="1">
-        <v>45941</v>
+        <v>45976</v>
       </c>
       <c r="D93" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E93">
-        <v>336.78</v>
+        <v>253.41</v>
       </c>
       <c r="F93" t="s">
         <v>29</v>
@@ -2589,19 +2589,19 @@
     </row>
     <row r="94" spans="1:7">
       <c r="A94">
-        <v>90009</v>
+        <v>90005</v>
       </c>
       <c r="B94">
         <v>810092</v>
       </c>
       <c r="C94" s="1">
-        <v>45664</v>
+        <v>45771</v>
       </c>
       <c r="D94" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E94">
-        <v>276.52</v>
+        <v>60.08</v>
       </c>
       <c r="F94" t="s">
         <v>29</v>
@@ -2612,19 +2612,19 @@
     </row>
     <row r="95" spans="1:7">
       <c r="A95">
-        <v>90011</v>
+        <v>90006</v>
       </c>
       <c r="B95">
         <v>810093</v>
       </c>
       <c r="C95" s="1">
-        <v>46112</v>
+        <v>45880</v>
       </c>
       <c r="D95" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E95">
-        <v>247.71</v>
+        <v>335.25</v>
       </c>
       <c r="F95" t="s">
         <v>29</v>
@@ -2635,19 +2635,19 @@
     </row>
     <row r="96" spans="1:7">
       <c r="A96">
-        <v>90006</v>
+        <v>90003</v>
       </c>
       <c r="B96">
         <v>810094</v>
       </c>
       <c r="C96" s="1">
-        <v>45680</v>
+        <v>45859</v>
       </c>
       <c r="D96" t="s">
         <v>25</v>
       </c>
       <c r="E96">
-        <v>184.73</v>
+        <v>340.54</v>
       </c>
       <c r="F96" t="s">
         <v>29</v>
@@ -2658,19 +2658,19 @@
     </row>
     <row r="97" spans="1:7">
       <c r="A97">
-        <v>90008</v>
+        <v>90002</v>
       </c>
       <c r="B97">
         <v>810095</v>
       </c>
       <c r="C97" s="1">
-        <v>45907</v>
+        <v>45857</v>
       </c>
       <c r="D97" t="s">
         <v>26</v>
       </c>
       <c r="E97">
-        <v>53.5</v>
+        <v>332.61</v>
       </c>
       <c r="F97" t="s">
         <v>29</v>
@@ -2681,42 +2681,42 @@
     </row>
     <row r="98" spans="1:7">
       <c r="A98">
-        <v>90009</v>
+        <v>90006</v>
       </c>
       <c r="B98">
         <v>810096</v>
       </c>
       <c r="C98" s="1">
-        <v>45765</v>
+        <v>46115</v>
       </c>
       <c r="D98" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E98">
-        <v>285.57</v>
+        <v>227.18</v>
       </c>
       <c r="F98" t="s">
         <v>29</v>
       </c>
       <c r="G98" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="99" spans="1:7">
       <c r="A99">
-        <v>90010</v>
+        <v>90007</v>
       </c>
       <c r="B99">
         <v>810097</v>
       </c>
       <c r="C99" s="1">
-        <v>45876</v>
+        <v>45983</v>
       </c>
       <c r="D99" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E99">
-        <v>189.05</v>
+        <v>231.73</v>
       </c>
       <c r="F99" t="s">
         <v>29</v>
@@ -2727,25 +2727,25 @@
     </row>
     <row r="100" spans="1:7">
       <c r="A100">
-        <v>90010</v>
+        <v>90002</v>
       </c>
       <c r="B100">
         <v>810098</v>
       </c>
       <c r="C100" s="1">
-        <v>46032</v>
+        <v>46053</v>
       </c>
       <c r="D100" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E100">
-        <v>202.09</v>
+        <v>163.31</v>
       </c>
       <c r="F100" t="s">
         <v>29</v>
       </c>
       <c r="G100" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="101" spans="1:7">
@@ -2756,13 +2756,13 @@
         <v>810099</v>
       </c>
       <c r="C101" s="1">
-        <v>45877</v>
+        <v>46122</v>
       </c>
       <c r="D101" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E101">
-        <v>121.51</v>
+        <v>298.32</v>
       </c>
       <c r="F101" t="s">
         <v>29</v>
@@ -2773,19 +2773,19 @@
     </row>
     <row r="102" spans="1:7">
       <c r="A102">
-        <v>90003</v>
+        <v>90008</v>
       </c>
       <c r="B102">
         <v>810100</v>
       </c>
       <c r="C102" s="1">
-        <v>45829</v>
+        <v>46083</v>
       </c>
       <c r="D102" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E102">
-        <v>195.38</v>
+        <v>115.09</v>
       </c>
       <c r="F102" t="s">
         <v>29</v>
@@ -2796,19 +2796,19 @@
     </row>
     <row r="103" spans="1:7">
       <c r="A103">
-        <v>90011</v>
+        <v>90004</v>
       </c>
       <c r="B103">
         <v>810101</v>
       </c>
       <c r="C103" s="1">
-        <v>46025</v>
+        <v>45945</v>
       </c>
       <c r="D103" t="s">
         <v>28</v>
       </c>
       <c r="E103">
-        <v>157.05</v>
+        <v>52.64</v>
       </c>
       <c r="F103" t="s">
         <v>29</v>
@@ -2819,19 +2819,19 @@
     </row>
     <row r="104" spans="1:7">
       <c r="A104">
-        <v>90006</v>
+        <v>90005</v>
       </c>
       <c r="B104">
         <v>810102</v>
       </c>
       <c r="C104" s="1">
-        <v>45869</v>
+        <v>45753</v>
       </c>
       <c r="D104" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E104">
-        <v>348.2</v>
+        <v>339.07</v>
       </c>
       <c r="F104" t="s">
         <v>29</v>
@@ -2842,42 +2842,42 @@
     </row>
     <row r="105" spans="1:7">
       <c r="A105">
-        <v>90008</v>
+        <v>90002</v>
       </c>
       <c r="B105">
         <v>810103</v>
       </c>
       <c r="C105" s="1">
-        <v>45852</v>
+        <v>46083</v>
       </c>
       <c r="D105" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E105">
-        <v>312.48</v>
+        <v>47.71</v>
       </c>
       <c r="F105" t="s">
         <v>29</v>
       </c>
       <c r="G105" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="106" spans="1:7">
       <c r="A106">
-        <v>90003</v>
+        <v>90008</v>
       </c>
       <c r="B106">
         <v>810104</v>
       </c>
       <c r="C106" s="1">
-        <v>45727</v>
+        <v>45966</v>
       </c>
       <c r="D106" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E106">
-        <v>307.85</v>
+        <v>82.31999999999999</v>
       </c>
       <c r="F106" t="s">
         <v>29</v>
@@ -2888,19 +2888,19 @@
     </row>
     <row r="107" spans="1:7">
       <c r="A107">
-        <v>90009</v>
+        <v>90007</v>
       </c>
       <c r="B107">
         <v>810105</v>
       </c>
       <c r="C107" s="1">
-        <v>45736</v>
+        <v>45963</v>
       </c>
       <c r="D107" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E107">
-        <v>178.16</v>
+        <v>130.22</v>
       </c>
       <c r="F107" t="s">
         <v>29</v>
@@ -2911,19 +2911,19 @@
     </row>
     <row r="108" spans="1:7">
       <c r="A108">
-        <v>90012</v>
+        <v>90008</v>
       </c>
       <c r="B108">
         <v>810106</v>
       </c>
       <c r="C108" s="1">
-        <v>45821</v>
+        <v>46001</v>
       </c>
       <c r="D108" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E108">
-        <v>81.41</v>
+        <v>200.13</v>
       </c>
       <c r="F108" t="s">
         <v>29</v>
@@ -2934,19 +2934,19 @@
     </row>
     <row r="109" spans="1:7">
       <c r="A109">
-        <v>90009</v>
+        <v>90012</v>
       </c>
       <c r="B109">
         <v>810107</v>
       </c>
       <c r="C109" s="1">
-        <v>45915</v>
+        <v>46021</v>
       </c>
       <c r="D109" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E109">
-        <v>30.95</v>
+        <v>248</v>
       </c>
       <c r="F109" t="s">
         <v>29</v>
@@ -2957,42 +2957,42 @@
     </row>
     <row r="110" spans="1:7">
       <c r="A110">
-        <v>90012</v>
+        <v>90002</v>
       </c>
       <c r="B110">
         <v>810108</v>
       </c>
       <c r="C110" s="1">
-        <v>45668</v>
+        <v>46061</v>
       </c>
       <c r="D110" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E110">
-        <v>57.99</v>
+        <v>211.08</v>
       </c>
       <c r="F110" t="s">
         <v>29</v>
       </c>
       <c r="G110" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="111" spans="1:7">
       <c r="A111">
-        <v>90003</v>
+        <v>90010</v>
       </c>
       <c r="B111">
         <v>810109</v>
       </c>
       <c r="C111" s="1">
-        <v>45772</v>
+        <v>45730</v>
       </c>
       <c r="D111" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E111">
-        <v>139.71</v>
+        <v>61.37</v>
       </c>
       <c r="F111" t="s">
         <v>29</v>
@@ -3003,88 +3003,88 @@
     </row>
     <row r="112" spans="1:7">
       <c r="A112">
-        <v>90011</v>
+        <v>90003</v>
       </c>
       <c r="B112">
         <v>810110</v>
       </c>
       <c r="C112" s="1">
-        <v>46095</v>
+        <v>46105</v>
       </c>
       <c r="D112" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E112">
-        <v>334.78</v>
+        <v>298.73</v>
       </c>
       <c r="F112" t="s">
         <v>29</v>
       </c>
       <c r="G112" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="113" spans="1:7">
       <c r="A113">
-        <v>90007</v>
+        <v>90006</v>
       </c>
       <c r="B113">
         <v>810111</v>
       </c>
       <c r="C113" s="1">
-        <v>45742</v>
+        <v>45747</v>
       </c>
       <c r="D113" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E113">
-        <v>271.39</v>
+        <v>299.41</v>
       </c>
       <c r="F113" t="s">
         <v>29</v>
       </c>
       <c r="G113" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="114" spans="1:7">
       <c r="A114">
-        <v>90002</v>
+        <v>90009</v>
       </c>
       <c r="B114">
         <v>810112</v>
       </c>
       <c r="C114" s="1">
-        <v>45757</v>
+        <v>46077</v>
       </c>
       <c r="D114" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E114">
-        <v>346.62</v>
+        <v>254</v>
       </c>
       <c r="F114" t="s">
         <v>29</v>
       </c>
       <c r="G114" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="115" spans="1:7">
       <c r="A115">
-        <v>90007</v>
+        <v>90001</v>
       </c>
       <c r="B115">
         <v>810113</v>
       </c>
       <c r="C115" s="1">
-        <v>45944</v>
+        <v>45709</v>
       </c>
       <c r="D115" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E115">
-        <v>306.37</v>
+        <v>189.59</v>
       </c>
       <c r="F115" t="s">
         <v>29</v>
@@ -3095,42 +3095,42 @@
     </row>
     <row r="116" spans="1:7">
       <c r="A116">
-        <v>90009</v>
+        <v>90007</v>
       </c>
       <c r="B116">
         <v>810114</v>
       </c>
       <c r="C116" s="1">
-        <v>46090</v>
+        <v>45898</v>
       </c>
       <c r="D116" t="s">
         <v>25</v>
       </c>
       <c r="E116">
-        <v>158.3</v>
+        <v>100.51</v>
       </c>
       <c r="F116" t="s">
         <v>29</v>
       </c>
       <c r="G116" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="117" spans="1:7">
       <c r="A117">
-        <v>90007</v>
+        <v>90002</v>
       </c>
       <c r="B117">
         <v>810115</v>
       </c>
       <c r="C117" s="1">
-        <v>45703</v>
+        <v>45947</v>
       </c>
       <c r="D117" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E117">
-        <v>314.27</v>
+        <v>187.82</v>
       </c>
       <c r="F117" t="s">
         <v>29</v>
@@ -3141,19 +3141,19 @@
     </row>
     <row r="118" spans="1:7">
       <c r="A118">
-        <v>90002</v>
+        <v>90010</v>
       </c>
       <c r="B118">
         <v>810116</v>
       </c>
       <c r="C118" s="1">
-        <v>45734</v>
+        <v>45800</v>
       </c>
       <c r="D118" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E118">
-        <v>322.74</v>
+        <v>242.3</v>
       </c>
       <c r="F118" t="s">
         <v>29</v>
@@ -3164,19 +3164,19 @@
     </row>
     <row r="119" spans="1:7">
       <c r="A119">
-        <v>90004</v>
+        <v>90001</v>
       </c>
       <c r="B119">
         <v>810117</v>
       </c>
       <c r="C119" s="1">
-        <v>45854</v>
+        <v>46025</v>
       </c>
       <c r="D119" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E119">
-        <v>301.25</v>
+        <v>303.94</v>
       </c>
       <c r="F119" t="s">
         <v>29</v>
@@ -3187,19 +3187,19 @@
     </row>
     <row r="120" spans="1:7">
       <c r="A120">
-        <v>90001</v>
+        <v>90002</v>
       </c>
       <c r="B120">
         <v>810118</v>
       </c>
       <c r="C120" s="1">
-        <v>45775</v>
+        <v>45837</v>
       </c>
       <c r="D120" t="s">
         <v>28</v>
       </c>
       <c r="E120">
-        <v>25.06</v>
+        <v>178.61</v>
       </c>
       <c r="F120" t="s">
         <v>29</v>
@@ -3210,19 +3210,19 @@
     </row>
     <row r="121" spans="1:7">
       <c r="A121">
-        <v>90010</v>
+        <v>90001</v>
       </c>
       <c r="B121">
         <v>810119</v>
       </c>
       <c r="C121" s="1">
-        <v>46081</v>
+        <v>45761</v>
       </c>
       <c r="D121" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E121">
-        <v>163.51</v>
+        <v>162.94</v>
       </c>
       <c r="F121" t="s">
         <v>29</v>
@@ -3233,19 +3233,19 @@
     </row>
     <row r="122" spans="1:7">
       <c r="A122">
-        <v>90005</v>
+        <v>90012</v>
       </c>
       <c r="B122">
         <v>810120</v>
       </c>
       <c r="C122" s="1">
-        <v>45895</v>
+        <v>45789</v>
       </c>
       <c r="D122" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E122">
-        <v>55.69</v>
+        <v>200.16</v>
       </c>
       <c r="F122" t="s">
         <v>29</v>
@@ -3256,42 +3256,42 @@
     </row>
     <row r="123" spans="1:7">
       <c r="A123">
-        <v>90009</v>
+        <v>90007</v>
       </c>
       <c r="B123">
         <v>810121</v>
       </c>
       <c r="C123" s="1">
-        <v>46030</v>
+        <v>46136</v>
       </c>
       <c r="D123" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E123">
-        <v>340.38</v>
+        <v>224.58</v>
       </c>
       <c r="F123" t="s">
         <v>29</v>
       </c>
       <c r="G123" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="124" spans="1:7">
       <c r="A124">
-        <v>90004</v>
+        <v>90007</v>
       </c>
       <c r="B124">
         <v>810122</v>
       </c>
       <c r="C124" s="1">
-        <v>45830</v>
+        <v>46133</v>
       </c>
       <c r="D124" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E124">
-        <v>128.04</v>
+        <v>87.97</v>
       </c>
       <c r="F124" t="s">
         <v>29</v>
@@ -3302,19 +3302,19 @@
     </row>
     <row r="125" spans="1:7">
       <c r="A125">
-        <v>90012</v>
+        <v>90003</v>
       </c>
       <c r="B125">
         <v>810123</v>
       </c>
       <c r="C125" s="1">
-        <v>45785</v>
+        <v>45945</v>
       </c>
       <c r="D125" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E125">
-        <v>306.35</v>
+        <v>129.37</v>
       </c>
       <c r="F125" t="s">
         <v>29</v>
@@ -3325,88 +3325,88 @@
     </row>
     <row r="126" spans="1:7">
       <c r="A126">
-        <v>90010</v>
+        <v>90009</v>
       </c>
       <c r="B126">
         <v>810124</v>
       </c>
       <c r="C126" s="1">
-        <v>45858</v>
+        <v>45853</v>
       </c>
       <c r="D126" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E126">
-        <v>211.14</v>
+        <v>270.4</v>
       </c>
       <c r="F126" t="s">
         <v>29</v>
       </c>
       <c r="G126" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="127" spans="1:7">
       <c r="A127">
-        <v>90002</v>
+        <v>90001</v>
       </c>
       <c r="B127">
         <v>810125</v>
       </c>
       <c r="C127" s="1">
-        <v>45848</v>
+        <v>45916</v>
       </c>
       <c r="D127" t="s">
         <v>26</v>
       </c>
       <c r="E127">
-        <v>122.15</v>
+        <v>86.34999999999999</v>
       </c>
       <c r="F127" t="s">
         <v>29</v>
       </c>
       <c r="G127" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="128" spans="1:7">
       <c r="A128">
-        <v>90008</v>
+        <v>90005</v>
       </c>
       <c r="B128">
         <v>810126</v>
       </c>
       <c r="C128" s="1">
-        <v>45821</v>
+        <v>45707</v>
       </c>
       <c r="D128" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E128">
-        <v>345.9</v>
+        <v>264.29</v>
       </c>
       <c r="F128" t="s">
         <v>29</v>
       </c>
       <c r="G128" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="129" spans="1:7">
       <c r="A129">
-        <v>90012</v>
+        <v>90010</v>
       </c>
       <c r="B129">
         <v>810127</v>
       </c>
       <c r="C129" s="1">
-        <v>46055</v>
+        <v>45855</v>
       </c>
       <c r="D129" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E129">
-        <v>30.82</v>
+        <v>310.32</v>
       </c>
       <c r="F129" t="s">
         <v>29</v>
@@ -3417,42 +3417,42 @@
     </row>
     <row r="130" spans="1:7">
       <c r="A130">
-        <v>90005</v>
+        <v>90002</v>
       </c>
       <c r="B130">
         <v>810128</v>
       </c>
       <c r="C130" s="1">
-        <v>45799</v>
+        <v>45779</v>
       </c>
       <c r="D130" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E130">
-        <v>52.12</v>
+        <v>224.54</v>
       </c>
       <c r="F130" t="s">
         <v>29</v>
       </c>
       <c r="G130" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="131" spans="1:7">
       <c r="A131">
-        <v>90009</v>
+        <v>90003</v>
       </c>
       <c r="B131">
         <v>810129</v>
       </c>
       <c r="C131" s="1">
-        <v>45821</v>
+        <v>45937</v>
       </c>
       <c r="D131" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E131">
-        <v>177.65</v>
+        <v>90.48</v>
       </c>
       <c r="F131" t="s">
         <v>29</v>
@@ -3469,88 +3469,88 @@
         <v>810130</v>
       </c>
       <c r="C132" s="1">
-        <v>45710</v>
+        <v>45712</v>
       </c>
       <c r="D132" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E132">
-        <v>259.69</v>
+        <v>174.05</v>
       </c>
       <c r="F132" t="s">
         <v>29</v>
       </c>
       <c r="G132" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="133" spans="1:7">
       <c r="A133">
-        <v>90005</v>
+        <v>90009</v>
       </c>
       <c r="B133">
         <v>810131</v>
       </c>
       <c r="C133" s="1">
-        <v>45742</v>
+        <v>45955</v>
       </c>
       <c r="D133" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E133">
-        <v>294.03</v>
+        <v>327.87</v>
       </c>
       <c r="F133" t="s">
         <v>29</v>
       </c>
       <c r="G133" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="134" spans="1:7">
       <c r="A134">
-        <v>90007</v>
+        <v>90010</v>
       </c>
       <c r="B134">
         <v>810132</v>
       </c>
       <c r="C134" s="1">
-        <v>45826</v>
+        <v>45739</v>
       </c>
       <c r="D134" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E134">
-        <v>126.89</v>
+        <v>317.73</v>
       </c>
       <c r="F134" t="s">
         <v>29</v>
       </c>
       <c r="G134" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="135" spans="1:7">
       <c r="A135">
-        <v>90010</v>
+        <v>90005</v>
       </c>
       <c r="B135">
         <v>810133</v>
       </c>
       <c r="C135" s="1">
-        <v>45893</v>
+        <v>45846</v>
       </c>
       <c r="D135" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E135">
-        <v>119.84</v>
+        <v>202.33</v>
       </c>
       <c r="F135" t="s">
         <v>29</v>
       </c>
       <c r="G135" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="136" spans="1:7">
@@ -3561,82 +3561,82 @@
         <v>810134</v>
       </c>
       <c r="C136" s="1">
-        <v>46094</v>
+        <v>45674</v>
       </c>
       <c r="D136" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E136">
-        <v>265.02</v>
+        <v>193.87</v>
       </c>
       <c r="F136" t="s">
         <v>29</v>
       </c>
       <c r="G136" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="137" spans="1:7">
       <c r="A137">
-        <v>90011</v>
+        <v>90007</v>
       </c>
       <c r="B137">
         <v>810135</v>
       </c>
       <c r="C137" s="1">
-        <v>45850</v>
+        <v>45753</v>
       </c>
       <c r="D137" t="s">
         <v>26</v>
       </c>
       <c r="E137">
-        <v>73.83</v>
+        <v>339.21</v>
       </c>
       <c r="F137" t="s">
         <v>29</v>
       </c>
       <c r="G137" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="138" spans="1:7">
       <c r="A138">
-        <v>90003</v>
+        <v>90006</v>
       </c>
       <c r="B138">
         <v>810136</v>
       </c>
       <c r="C138" s="1">
-        <v>46006</v>
+        <v>46059</v>
       </c>
       <c r="D138" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E138">
-        <v>122.1</v>
+        <v>252.81</v>
       </c>
       <c r="F138" t="s">
         <v>29</v>
       </c>
       <c r="G138" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="139" spans="1:7">
       <c r="A139">
-        <v>90009</v>
+        <v>90008</v>
       </c>
       <c r="B139">
         <v>810137</v>
       </c>
       <c r="C139" s="1">
-        <v>45934</v>
+        <v>45697</v>
       </c>
       <c r="D139" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E139">
-        <v>204.51</v>
+        <v>139.24</v>
       </c>
       <c r="F139" t="s">
         <v>29</v>
@@ -3647,19 +3647,19 @@
     </row>
     <row r="140" spans="1:7">
       <c r="A140">
-        <v>90009</v>
+        <v>90004</v>
       </c>
       <c r="B140">
         <v>810138</v>
       </c>
       <c r="C140" s="1">
-        <v>45943</v>
+        <v>45753</v>
       </c>
       <c r="D140" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E140">
-        <v>150.12</v>
+        <v>310</v>
       </c>
       <c r="F140" t="s">
         <v>29</v>
@@ -3670,25 +3670,25 @@
     </row>
     <row r="141" spans="1:7">
       <c r="A141">
-        <v>90010</v>
+        <v>90007</v>
       </c>
       <c r="B141">
         <v>810139</v>
       </c>
       <c r="C141" s="1">
-        <v>46009</v>
+        <v>45786</v>
       </c>
       <c r="D141" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E141">
-        <v>146.13</v>
+        <v>324.39</v>
       </c>
       <c r="F141" t="s">
         <v>29</v>
       </c>
       <c r="G141" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="142" spans="1:7">
@@ -3699,82 +3699,82 @@
         <v>810140</v>
       </c>
       <c r="C142" s="1">
-        <v>46003</v>
+        <v>45789</v>
       </c>
       <c r="D142" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E142">
-        <v>220.88</v>
+        <v>101.81</v>
       </c>
       <c r="F142" t="s">
         <v>29</v>
       </c>
       <c r="G142" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="143" spans="1:7">
       <c r="A143">
-        <v>90008</v>
+        <v>90011</v>
       </c>
       <c r="B143">
         <v>810141</v>
       </c>
       <c r="C143" s="1">
-        <v>45665</v>
+        <v>45804</v>
       </c>
       <c r="D143" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E143">
-        <v>227.68</v>
+        <v>174.4</v>
       </c>
       <c r="F143" t="s">
         <v>29</v>
       </c>
       <c r="G143" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="144" spans="1:7">
       <c r="A144">
-        <v>90007</v>
+        <v>90008</v>
       </c>
       <c r="B144">
         <v>810142</v>
       </c>
       <c r="C144" s="1">
-        <v>45950</v>
+        <v>46118</v>
       </c>
       <c r="D144" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E144">
-        <v>33.18</v>
+        <v>139.73</v>
       </c>
       <c r="F144" t="s">
         <v>29</v>
       </c>
       <c r="G144" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="145" spans="1:7">
       <c r="A145">
-        <v>90009</v>
+        <v>90001</v>
       </c>
       <c r="B145">
         <v>810143</v>
       </c>
       <c r="C145" s="1">
-        <v>46014</v>
+        <v>45742</v>
       </c>
       <c r="D145" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E145">
-        <v>32.73</v>
+        <v>59.45</v>
       </c>
       <c r="F145" t="s">
         <v>29</v>
@@ -3785,42 +3785,42 @@
     </row>
     <row r="146" spans="1:7">
       <c r="A146">
-        <v>90001</v>
+        <v>90003</v>
       </c>
       <c r="B146">
         <v>810144</v>
       </c>
       <c r="C146" s="1">
-        <v>45748</v>
+        <v>45827</v>
       </c>
       <c r="D146" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E146">
-        <v>58.54</v>
+        <v>336.94</v>
       </c>
       <c r="F146" t="s">
         <v>29</v>
       </c>
       <c r="G146" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="147" spans="1:7">
       <c r="A147">
-        <v>90011</v>
+        <v>90010</v>
       </c>
       <c r="B147">
         <v>810145</v>
       </c>
       <c r="C147" s="1">
-        <v>45722</v>
+        <v>45987</v>
       </c>
       <c r="D147" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E147">
-        <v>23.06</v>
+        <v>346.89</v>
       </c>
       <c r="F147" t="s">
         <v>29</v>
@@ -3831,42 +3831,42 @@
     </row>
     <row r="148" spans="1:7">
       <c r="A148">
-        <v>90004</v>
+        <v>90012</v>
       </c>
       <c r="B148">
         <v>810146</v>
       </c>
       <c r="C148" s="1">
-        <v>46110</v>
+        <v>45892</v>
       </c>
       <c r="D148" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E148">
-        <v>185.23</v>
+        <v>237.14</v>
       </c>
       <c r="F148" t="s">
         <v>29</v>
       </c>
       <c r="G148" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="149" spans="1:7">
       <c r="A149">
-        <v>90008</v>
+        <v>90001</v>
       </c>
       <c r="B149">
         <v>810147</v>
       </c>
       <c r="C149" s="1">
-        <v>45769</v>
+        <v>46126</v>
       </c>
       <c r="D149" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E149">
-        <v>236.69</v>
+        <v>173.37</v>
       </c>
       <c r="F149" t="s">
         <v>29</v>
@@ -3877,65 +3877,65 @@
     </row>
     <row r="150" spans="1:7">
       <c r="A150">
-        <v>90009</v>
+        <v>90010</v>
       </c>
       <c r="B150">
         <v>810148</v>
       </c>
       <c r="C150" s="1">
-        <v>45968</v>
+        <v>45958</v>
       </c>
       <c r="D150" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E150">
-        <v>142.26</v>
+        <v>115.5</v>
       </c>
       <c r="F150" t="s">
         <v>29</v>
       </c>
       <c r="G150" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="151" spans="1:7">
       <c r="A151">
-        <v>90012</v>
+        <v>90001</v>
       </c>
       <c r="B151">
         <v>810149</v>
       </c>
       <c r="C151" s="1">
-        <v>45935</v>
+        <v>45687</v>
       </c>
       <c r="D151" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E151">
-        <v>61.28</v>
+        <v>310.72</v>
       </c>
       <c r="F151" t="s">
         <v>29</v>
       </c>
       <c r="G151" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="152" spans="1:7">
       <c r="A152">
-        <v>90006</v>
+        <v>90011</v>
       </c>
       <c r="B152">
         <v>810150</v>
       </c>
       <c r="C152" s="1">
-        <v>45972</v>
+        <v>45946</v>
       </c>
       <c r="D152" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E152">
-        <v>181.5</v>
+        <v>269.04</v>
       </c>
       <c r="F152" t="s">
         <v>29</v>
@@ -3946,65 +3946,65 @@
     </row>
     <row r="153" spans="1:7">
       <c r="A153">
-        <v>90011</v>
+        <v>90003</v>
       </c>
       <c r="B153">
         <v>810151</v>
       </c>
       <c r="C153" s="1">
-        <v>45805</v>
+        <v>46044</v>
       </c>
       <c r="D153" t="s">
         <v>26</v>
       </c>
       <c r="E153">
-        <v>201.22</v>
+        <v>210.9</v>
       </c>
       <c r="F153" t="s">
         <v>29</v>
       </c>
       <c r="G153" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="154" spans="1:7">
       <c r="A154">
-        <v>90007</v>
+        <v>90009</v>
       </c>
       <c r="B154">
         <v>810152</v>
       </c>
       <c r="C154" s="1">
-        <v>46001</v>
+        <v>45812</v>
       </c>
       <c r="D154" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E154">
-        <v>152.05</v>
+        <v>339.39</v>
       </c>
       <c r="F154" t="s">
         <v>29</v>
       </c>
       <c r="G154" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="155" spans="1:7">
       <c r="A155">
-        <v>90003</v>
+        <v>90005</v>
       </c>
       <c r="B155">
         <v>810153</v>
       </c>
       <c r="C155" s="1">
-        <v>46131</v>
+        <v>45904</v>
       </c>
       <c r="D155" t="s">
         <v>28</v>
       </c>
       <c r="E155">
-        <v>55.08</v>
+        <v>21.1</v>
       </c>
       <c r="F155" t="s">
         <v>29</v>
@@ -4015,42 +4015,42 @@
     </row>
     <row r="156" spans="1:7">
       <c r="A156">
-        <v>90012</v>
+        <v>90008</v>
       </c>
       <c r="B156">
         <v>810154</v>
       </c>
       <c r="C156" s="1">
-        <v>45687</v>
+        <v>45719</v>
       </c>
       <c r="D156" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E156">
-        <v>322.98</v>
+        <v>47.94</v>
       </c>
       <c r="F156" t="s">
         <v>29</v>
       </c>
       <c r="G156" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="157" spans="1:7">
       <c r="A157">
-        <v>90004</v>
+        <v>90010</v>
       </c>
       <c r="B157">
         <v>810155</v>
       </c>
       <c r="C157" s="1">
-        <v>45786</v>
+        <v>45955</v>
       </c>
       <c r="D157" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E157">
-        <v>175.33</v>
+        <v>135.36</v>
       </c>
       <c r="F157" t="s">
         <v>29</v>
@@ -4061,19 +4061,19 @@
     </row>
     <row r="158" spans="1:7">
       <c r="A158">
-        <v>90011</v>
+        <v>90010</v>
       </c>
       <c r="B158">
         <v>810156</v>
       </c>
       <c r="C158" s="1">
-        <v>45777</v>
+        <v>46035</v>
       </c>
       <c r="D158" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E158">
-        <v>309.28</v>
+        <v>166.3</v>
       </c>
       <c r="F158" t="s">
         <v>29</v>
@@ -4084,19 +4084,19 @@
     </row>
     <row r="159" spans="1:7">
       <c r="A159">
-        <v>90008</v>
+        <v>90007</v>
       </c>
       <c r="B159">
         <v>810157</v>
       </c>
       <c r="C159" s="1">
-        <v>45873</v>
+        <v>45695</v>
       </c>
       <c r="D159" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E159">
-        <v>322.48</v>
+        <v>160.24</v>
       </c>
       <c r="F159" t="s">
         <v>29</v>
@@ -4107,65 +4107,65 @@
     </row>
     <row r="160" spans="1:7">
       <c r="A160">
-        <v>90004</v>
+        <v>90002</v>
       </c>
       <c r="B160">
         <v>810158</v>
       </c>
       <c r="C160" s="1">
-        <v>45987</v>
+        <v>45683</v>
       </c>
       <c r="D160" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E160">
-        <v>107.84</v>
+        <v>22.63</v>
       </c>
       <c r="F160" t="s">
         <v>29</v>
       </c>
       <c r="G160" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="161" spans="1:7">
       <c r="A161">
-        <v>90007</v>
+        <v>90008</v>
       </c>
       <c r="B161">
         <v>810159</v>
       </c>
       <c r="C161" s="1">
-        <v>46112</v>
+        <v>45809</v>
       </c>
       <c r="D161" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E161">
-        <v>183.82</v>
+        <v>226.63</v>
       </c>
       <c r="F161" t="s">
         <v>29</v>
       </c>
       <c r="G161" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="162" spans="1:7">
       <c r="A162">
-        <v>90008</v>
+        <v>90002</v>
       </c>
       <c r="B162">
         <v>810160</v>
       </c>
       <c r="C162" s="1">
-        <v>45894</v>
+        <v>45951</v>
       </c>
       <c r="D162" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E162">
-        <v>74.34999999999999</v>
+        <v>70.16</v>
       </c>
       <c r="F162" t="s">
         <v>29</v>
@@ -4176,42 +4176,42 @@
     </row>
     <row r="163" spans="1:7">
       <c r="A163">
-        <v>90007</v>
+        <v>90008</v>
       </c>
       <c r="B163">
         <v>810161</v>
       </c>
       <c r="C163" s="1">
-        <v>45720</v>
+        <v>45807</v>
       </c>
       <c r="D163" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E163">
-        <v>294.33</v>
+        <v>150.39</v>
       </c>
       <c r="F163" t="s">
         <v>29</v>
       </c>
       <c r="G163" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="164" spans="1:7">
       <c r="A164">
-        <v>90012</v>
+        <v>90011</v>
       </c>
       <c r="B164">
         <v>810162</v>
       </c>
       <c r="C164" s="1">
-        <v>45838</v>
+        <v>45679</v>
       </c>
       <c r="D164" t="s">
         <v>27</v>
       </c>
       <c r="E164">
-        <v>55.69</v>
+        <v>178.82</v>
       </c>
       <c r="F164" t="s">
         <v>29</v>
@@ -4228,13 +4228,13 @@
         <v>810163</v>
       </c>
       <c r="C165" s="1">
-        <v>45729</v>
+        <v>45940</v>
       </c>
       <c r="D165" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E165">
-        <v>259.31</v>
+        <v>258.67</v>
       </c>
       <c r="F165" t="s">
         <v>29</v>
@@ -4245,65 +4245,65 @@
     </row>
     <row r="166" spans="1:7">
       <c r="A166">
-        <v>90002</v>
+        <v>90011</v>
       </c>
       <c r="B166">
         <v>810164</v>
       </c>
       <c r="C166" s="1">
-        <v>45906</v>
+        <v>46115</v>
       </c>
       <c r="D166" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E166">
-        <v>342.7</v>
+        <v>134.93</v>
       </c>
       <c r="F166" t="s">
         <v>29</v>
       </c>
       <c r="G166" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="167" spans="1:7">
       <c r="A167">
-        <v>90007</v>
+        <v>90001</v>
       </c>
       <c r="B167">
         <v>810165</v>
       </c>
       <c r="C167" s="1">
-        <v>46087</v>
+        <v>45976</v>
       </c>
       <c r="D167" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E167">
-        <v>238.86</v>
+        <v>105.13</v>
       </c>
       <c r="F167" t="s">
         <v>29</v>
       </c>
       <c r="G167" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="168" spans="1:7">
       <c r="A168">
-        <v>90008</v>
+        <v>90004</v>
       </c>
       <c r="B168">
         <v>810166</v>
       </c>
       <c r="C168" s="1">
-        <v>45931</v>
+        <v>45773</v>
       </c>
       <c r="D168" t="s">
         <v>26</v>
       </c>
       <c r="E168">
-        <v>114.51</v>
+        <v>150.7</v>
       </c>
       <c r="F168" t="s">
         <v>29</v>
@@ -4314,88 +4314,88 @@
     </row>
     <row r="169" spans="1:7">
       <c r="A169">
-        <v>90012</v>
+        <v>90003</v>
       </c>
       <c r="B169">
         <v>810167</v>
       </c>
       <c r="C169" s="1">
-        <v>45964</v>
+        <v>45961</v>
       </c>
       <c r="D169" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E169">
-        <v>252.27</v>
+        <v>203.43</v>
       </c>
       <c r="F169" t="s">
         <v>29</v>
       </c>
       <c r="G169" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="170" spans="1:7">
       <c r="A170">
-        <v>90006</v>
+        <v>90003</v>
       </c>
       <c r="B170">
         <v>810168</v>
       </c>
       <c r="C170" s="1">
-        <v>45748</v>
+        <v>45862</v>
       </c>
       <c r="D170" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E170">
-        <v>314.95</v>
+        <v>144.3</v>
       </c>
       <c r="F170" t="s">
         <v>29</v>
       </c>
       <c r="G170" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="171" spans="1:7">
       <c r="A171">
-        <v>90002</v>
+        <v>90005</v>
       </c>
       <c r="B171">
         <v>810169</v>
       </c>
       <c r="C171" s="1">
-        <v>46107</v>
+        <v>46053</v>
       </c>
       <c r="D171" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E171">
-        <v>113.28</v>
+        <v>154.95</v>
       </c>
       <c r="F171" t="s">
         <v>29</v>
       </c>
       <c r="G171" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="172" spans="1:7">
       <c r="A172">
-        <v>90003</v>
+        <v>90005</v>
       </c>
       <c r="B172">
         <v>810170</v>
       </c>
       <c r="C172" s="1">
-        <v>45809</v>
+        <v>45742</v>
       </c>
       <c r="D172" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E172">
-        <v>312.14</v>
+        <v>266.7</v>
       </c>
       <c r="F172" t="s">
         <v>29</v>
@@ -4406,65 +4406,65 @@
     </row>
     <row r="173" spans="1:7">
       <c r="A173">
-        <v>90007</v>
+        <v>90012</v>
       </c>
       <c r="B173">
         <v>810171</v>
       </c>
       <c r="C173" s="1">
-        <v>46087</v>
+        <v>45830</v>
       </c>
       <c r="D173" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E173">
-        <v>33.99</v>
+        <v>60.18</v>
       </c>
       <c r="F173" t="s">
         <v>29</v>
       </c>
       <c r="G173" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="174" spans="1:7">
       <c r="A174">
-        <v>90010</v>
+        <v>90009</v>
       </c>
       <c r="B174">
         <v>810172</v>
       </c>
       <c r="C174" s="1">
-        <v>45689</v>
+        <v>45953</v>
       </c>
       <c r="D174" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E174">
-        <v>251.22</v>
+        <v>148.26</v>
       </c>
       <c r="F174" t="s">
         <v>29</v>
       </c>
       <c r="G174" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="175" spans="1:7">
       <c r="A175">
-        <v>90003</v>
+        <v>90001</v>
       </c>
       <c r="B175">
         <v>810173</v>
       </c>
       <c r="C175" s="1">
-        <v>45920</v>
+        <v>46141</v>
       </c>
       <c r="D175" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E175">
-        <v>291.68</v>
+        <v>88.31</v>
       </c>
       <c r="F175" t="s">
         <v>29</v>
@@ -4481,13 +4481,13 @@
         <v>810174</v>
       </c>
       <c r="C176" s="1">
-        <v>45764</v>
+        <v>45838</v>
       </c>
       <c r="D176" t="s">
         <v>27</v>
       </c>
       <c r="E176">
-        <v>89.01000000000001</v>
+        <v>318.08</v>
       </c>
       <c r="F176" t="s">
         <v>29</v>
@@ -4498,19 +4498,19 @@
     </row>
     <row r="177" spans="1:7">
       <c r="A177">
-        <v>90009</v>
+        <v>90003</v>
       </c>
       <c r="B177">
         <v>810175</v>
       </c>
       <c r="C177" s="1">
-        <v>46007</v>
+        <v>45694</v>
       </c>
       <c r="D177" t="s">
         <v>26</v>
       </c>
       <c r="E177">
-        <v>65.20999999999999</v>
+        <v>94.63</v>
       </c>
       <c r="F177" t="s">
         <v>29</v>
@@ -4521,25 +4521,25 @@
     </row>
     <row r="178" spans="1:7">
       <c r="A178">
-        <v>90008</v>
+        <v>90001</v>
       </c>
       <c r="B178">
         <v>810176</v>
       </c>
       <c r="C178" s="1">
-        <v>45902</v>
+        <v>45680</v>
       </c>
       <c r="D178" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E178">
-        <v>207.77</v>
+        <v>131.17</v>
       </c>
       <c r="F178" t="s">
         <v>29</v>
       </c>
       <c r="G178" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="179" spans="1:7">
@@ -4550,36 +4550,36 @@
         <v>810177</v>
       </c>
       <c r="C179" s="1">
-        <v>46071</v>
+        <v>45991</v>
       </c>
       <c r="D179" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E179">
-        <v>141.74</v>
+        <v>265.33</v>
       </c>
       <c r="F179" t="s">
         <v>29</v>
       </c>
       <c r="G179" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="180" spans="1:7">
       <c r="A180">
-        <v>90001</v>
+        <v>90003</v>
       </c>
       <c r="B180">
         <v>810178</v>
       </c>
       <c r="C180" s="1">
-        <v>45836</v>
+        <v>45828</v>
       </c>
       <c r="D180" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E180">
-        <v>313.02</v>
+        <v>150.56</v>
       </c>
       <c r="F180" t="s">
         <v>29</v>
@@ -4590,19 +4590,19 @@
     </row>
     <row r="181" spans="1:7">
       <c r="A181">
-        <v>90002</v>
+        <v>90005</v>
       </c>
       <c r="B181">
         <v>810179</v>
       </c>
       <c r="C181" s="1">
-        <v>46117</v>
+        <v>45752</v>
       </c>
       <c r="D181" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E181">
-        <v>297.54</v>
+        <v>277.73</v>
       </c>
       <c r="F181" t="s">
         <v>29</v>
@@ -4622,7 +4622,7 @@
         <v>7</v>
       </c>
       <c r="D182" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E182">
         <v>20</v>
@@ -4645,7 +4645,7 @@
         <v>8</v>
       </c>
       <c r="D183" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E183">
         <v>23</v>
@@ -4668,7 +4668,7 @@
         <v>9</v>
       </c>
       <c r="D184" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E184">
         <v>26</v>
@@ -4691,7 +4691,7 @@
         <v>10</v>
       </c>
       <c r="D185" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E185">
         <v>29</v>
@@ -4714,7 +4714,7 @@
         <v>11</v>
       </c>
       <c r="D186" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E186">
         <v>32</v>
@@ -4737,7 +4737,7 @@
         <v>12</v>
       </c>
       <c r="D187" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E187">
         <v>35</v>
@@ -4760,7 +4760,7 @@
         <v>13</v>
       </c>
       <c r="D188" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E188">
         <v>38</v>
@@ -4783,7 +4783,7 @@
         <v>14</v>
       </c>
       <c r="D189" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E189">
         <v>41</v>
@@ -4806,7 +4806,7 @@
         <v>15</v>
       </c>
       <c r="D190" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E190">
         <v>44</v>
@@ -4829,7 +4829,7 @@
         <v>16</v>
       </c>
       <c r="D191" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E191">
         <v>47</v>
@@ -4852,7 +4852,7 @@
         <v>17</v>
       </c>
       <c r="D192" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E192">
         <v>50</v>
@@ -4875,7 +4875,7 @@
         <v>18</v>
       </c>
       <c r="D193" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E193">
         <v>53</v>
@@ -4898,7 +4898,7 @@
         <v>19</v>
       </c>
       <c r="D194" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E194">
         <v>56</v>
@@ -4921,7 +4921,7 @@
         <v>20</v>
       </c>
       <c r="D195" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E195">
         <v>59</v>
@@ -4944,7 +4944,7 @@
         <v>21</v>
       </c>
       <c r="D196" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E196">
         <v>62</v>
@@ -4967,7 +4967,7 @@
         <v>22</v>
       </c>
       <c r="D197" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E197">
         <v>65</v>
@@ -4990,7 +4990,7 @@
         <v>23</v>
       </c>
       <c r="D198" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E198">
         <v>55.01</v>
@@ -5013,7 +5013,7 @@
         <v>24</v>
       </c>
       <c r="D199" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E199">
         <v>12.34</v>
@@ -5036,7 +5036,7 @@
         <v>24</v>
       </c>
       <c r="D200" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E200">
         <v>12.34</v>
@@ -5059,7 +5059,7 @@
         <v>24</v>
       </c>
       <c r="D201" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E201">
         <v>12.34</v>
@@ -5082,7 +5082,7 @@
         <v>24</v>
       </c>
       <c r="D202" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E202">
         <v>12.34</v>

</xml_diff>